<commit_message>
Refactor KPI modules: shared utils, fix NaN formatting and GDS Incentive YoY bug
- Add utils.py with shared format_number and format_percentage to eliminate
  copy-paste across kpi.py, kpi_rev.py, and kpi_month.py
- Fix NaN-safe YoY formatting in kpi.py and kpi_month.py (was producing "nan%"
  strings; now returns empty string via format_percentage)
- Fix typo df_pricelince -> df_priceline in kpi.py and kpi_rev.py
- Fix bug in summary_table_actual.py: GDS Incentive "Reporting Week" was
  comparing CW vs PW (not YoY), and "Previous Week" was always 0% (pct(pw, pw));
  corrected to use inc_cwly and inc_pwly for proper year-over-year comparison
- Remove dead commented-out code in kpi.py, kpi_rev.py, kpi_month.py

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/code/df_dau_converison.xlsx
+++ b/code/df_dau_converison.xlsx
@@ -537,676 +537,676 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>15286</v>
+        <v>15906</v>
       </c>
       <c r="B2" t="n">
-        <v>7108</v>
+        <v>8033</v>
       </c>
       <c r="C2" t="n">
-        <v>15547</v>
+        <v>14970</v>
       </c>
       <c r="D2" t="n">
-        <v>6598</v>
+        <v>6873</v>
       </c>
       <c r="E2" t="n">
-        <v>293005</v>
+        <v>323881</v>
       </c>
       <c r="F2" t="n">
-        <v>141608</v>
+        <v>156377</v>
       </c>
       <c r="G2" t="n">
-        <v>2195</v>
+        <v>2319</v>
       </c>
       <c r="H2" t="n">
-        <v>1315</v>
+        <v>1380</v>
       </c>
       <c r="I2" t="n">
-        <v>2198</v>
+        <v>2149</v>
       </c>
       <c r="J2" t="n">
-        <v>1210</v>
+        <v>1295</v>
       </c>
       <c r="K2" t="n">
-        <v>66.92015209125475</v>
+        <v>68.04347826086956</v>
       </c>
       <c r="L2" t="n">
-        <v>81.65289256198346</v>
+        <v>65.94594594594594</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>115.1%</t>
+          <t>98.0%</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>135.6%</t>
+          <t>117.8%</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>106.9%</t>
+          <t>107.1%</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.1435954468140782</v>
+        <v>0.1457940399849114</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.1850028137310073</v>
+        <v>0.1717913606373709</v>
       </c>
       <c r="R2" t="n">
-        <v>0.1413777577667717</v>
+        <v>0.1435537742150969</v>
       </c>
       <c r="S2" t="n">
-        <v>0.1833889057290088</v>
+        <v>0.1884184490033464</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>-22.4%</t>
+          <t>-15.1%</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>-22.9%</t>
+          <t>-23.8%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>870374</v>
+        <v>898231</v>
       </c>
       <c r="B3" t="n">
-        <v>824484</v>
+        <v>847197</v>
       </c>
       <c r="C3" t="n">
-        <v>899761</v>
+        <v>852626</v>
       </c>
       <c r="D3" t="n">
-        <v>817301</v>
+        <v>815315</v>
       </c>
       <c r="E3" t="n">
-        <v>17726467</v>
+        <v>19485347</v>
       </c>
       <c r="F3" t="n">
-        <v>17464497</v>
+        <v>19123403</v>
       </c>
       <c r="G3" t="n">
-        <v>48009</v>
+        <v>49185</v>
       </c>
       <c r="H3" t="n">
-        <v>50272</v>
+        <v>51457</v>
       </c>
       <c r="I3" t="n">
-        <v>48441</v>
+        <v>44937</v>
       </c>
       <c r="J3" t="n">
-        <v>51731</v>
+        <v>48338</v>
       </c>
       <c r="K3" t="n">
-        <v>-4.501511775938893</v>
+        <v>-4.4153370775599</v>
       </c>
       <c r="L3" t="n">
-        <v>-6.359822930157932</v>
+        <v>-7.035872398527044</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>10.1%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>1.9%</t>
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.05515904657078451</v>
+        <v>0.05475762916220883</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.06097389397489824</v>
+        <v>0.06073793934586643</v>
       </c>
       <c r="R3" t="n">
-        <v>0.05383763021513491</v>
+        <v>0.05270423374375165</v>
       </c>
       <c r="S3" t="n">
-        <v>0.06329491827368375</v>
+        <v>0.05928751464158025</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>-9.5%</t>
+          <t>-9.8%</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>-14.9%</t>
+          <t>-11.1%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>157594</v>
+        <v>157001</v>
       </c>
       <c r="B4" t="n">
-        <v>144933</v>
+        <v>151964</v>
       </c>
       <c r="C4" t="n">
-        <v>154740</v>
+        <v>147261</v>
       </c>
       <c r="D4" t="n">
-        <v>142278</v>
+        <v>140849</v>
       </c>
       <c r="E4" t="n">
-        <v>3095341</v>
+        <v>3399603</v>
       </c>
       <c r="F4" t="n">
-        <v>3027056</v>
+        <v>3318561</v>
       </c>
       <c r="G4" t="n">
-        <v>10445</v>
+        <v>10575</v>
       </c>
       <c r="H4" t="n">
-        <v>10230</v>
+        <v>10659</v>
       </c>
       <c r="I4" t="n">
-        <v>10106</v>
+        <v>9521</v>
       </c>
       <c r="J4" t="n">
-        <v>10454</v>
+        <v>9730</v>
       </c>
       <c r="K4" t="n">
-        <v>2.101661779081132</v>
+        <v>-0.7880664227413403</v>
       </c>
       <c r="L4" t="n">
-        <v>-3.328869332312989</v>
+        <v>-2.147995889003085</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>8.7%</t>
+          <t>3.3%</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>8.8%</t>
+          <t>4.6%</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2.3%</t>
+          <t>2.4%</t>
         </is>
       </c>
       <c r="P4" t="n">
-        <v>0.06627790398111603</v>
+        <v>0.06735625887733199</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.07058433897042081</v>
+        <v>0.07014161248716802</v>
       </c>
       <c r="R4" t="n">
-        <v>0.06530955150575159</v>
+        <v>0.06465391379930871</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0734758711817709</v>
+        <v>0.06908107263807339</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>-6.1%</t>
+          <t>-4.0%</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>-11.1%</t>
+          <t>-6.4%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>563868</v>
+        <v>550297</v>
       </c>
       <c r="B5" t="n">
-        <v>397907</v>
+        <v>448813</v>
       </c>
       <c r="C5" t="n">
-        <v>559369</v>
+        <v>518990</v>
       </c>
       <c r="D5" t="n">
-        <v>397120</v>
+        <v>388345</v>
       </c>
       <c r="E5" t="n">
-        <v>11107393</v>
+        <v>12176680</v>
       </c>
       <c r="F5" t="n">
-        <v>7753845</v>
+        <v>8584476</v>
       </c>
       <c r="G5" t="n">
-        <v>21045</v>
+        <v>21032</v>
       </c>
       <c r="H5" t="n">
-        <v>16554</v>
+        <v>18295</v>
       </c>
       <c r="I5" t="n">
-        <v>21610</v>
+        <v>18953</v>
       </c>
       <c r="J5" t="n">
-        <v>16717</v>
+        <v>15814</v>
       </c>
       <c r="K5" t="n">
-        <v>27.12939470822761</v>
+        <v>14.96037168625308</v>
       </c>
       <c r="L5" t="n">
-        <v>29.26960579051265</v>
+        <v>19.84950044264575</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>40.9%</t>
+          <t>33.6%</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>43.3%</t>
+          <t>41.8%</t>
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.03732256485560451</v>
+        <v>0.03821936154476582</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.04160268605478164</v>
+        <v>0.0407630795008166</v>
       </c>
       <c r="R5" t="n">
-        <v>0.03863281662015593</v>
+        <v>0.03651900807337329</v>
       </c>
       <c r="S5" t="n">
-        <v>0.04209558823529412</v>
+        <v>0.04072152338770938</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
+          <t>-6.2%</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
           <t>-10.3%</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>-8.2%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>254673</v>
+        <v>268940</v>
       </c>
       <c r="B6" t="n">
-        <v>255463</v>
+        <v>296377</v>
       </c>
       <c r="C6" t="n">
-        <v>251330</v>
+        <v>246977</v>
       </c>
       <c r="D6" t="n">
-        <v>225836</v>
+        <v>272244</v>
       </c>
       <c r="E6" t="n">
-        <v>4924084</v>
+        <v>5440001</v>
       </c>
       <c r="F6" t="n">
-        <v>4663901</v>
+        <v>5227645</v>
       </c>
       <c r="G6" t="n">
-        <v>3052</v>
+        <v>3209</v>
       </c>
       <c r="H6" t="n">
-        <v>3560</v>
+        <v>3807</v>
       </c>
       <c r="I6" t="n">
-        <v>3154</v>
+        <v>2864</v>
       </c>
       <c r="J6" t="n">
-        <v>3260</v>
+        <v>3603</v>
       </c>
       <c r="K6" t="n">
-        <v>-14.26966292134831</v>
+        <v>-15.70790648804833</v>
       </c>
       <c r="L6" t="n">
-        <v>-3.251533742331292</v>
+        <v>-20.51068553982792</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>-0.3%</t>
+          <t>-9.3%</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>11.3%</t>
+          <t>-9.3%</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>5.6%</t>
+          <t>4.1%</t>
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.01198399516242397</v>
+        <v>0.01193202944894772</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.01393548185060067</v>
+        <v>0.01284512630872166</v>
       </c>
       <c r="R6" t="n">
-        <v>0.01254923805355509</v>
+        <v>0.01159622151050503</v>
       </c>
       <c r="S6" t="n">
-        <v>0.01443525390106095</v>
+        <v>0.0132344514479658</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>-14.0%</t>
+          <t>-7.1%</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>-13.1%</t>
+          <t>-12.4%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>650</v>
+        <v>592</v>
       </c>
       <c r="B7" t="n">
-        <v>564</v>
+        <v>620</v>
       </c>
       <c r="C7" t="n">
-        <v>678</v>
+        <v>525</v>
       </c>
       <c r="D7" t="n">
-        <v>463</v>
+        <v>577</v>
       </c>
       <c r="E7" t="n">
-        <v>12985</v>
+        <v>14102</v>
       </c>
       <c r="F7" t="n">
-        <v>9651</v>
+        <v>10843</v>
       </c>
       <c r="G7" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="H7" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="I7" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="J7" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="K7" t="n">
-        <v>-4.545454545454541</v>
+        <v>6.25</v>
       </c>
       <c r="L7" t="n">
-        <v>-28.57142857142857</v>
+        <v>-33.33333333333334</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>-4.5%</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>46.4%</t>
+          <t>-9.0%</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>34.5%</t>
+          <t>30.1%</t>
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.03230769230769231</v>
+        <v>0.05743243243243244</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.03900709219858156</v>
+        <v>0.05161290322580645</v>
       </c>
       <c r="R7" t="n">
-        <v>0.03687315634218289</v>
+        <v>0.02285714285714286</v>
       </c>
       <c r="S7" t="n">
-        <v>0.0755939524838013</v>
+        <v>0.03119584055459272</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>-17.2%</t>
+          <t>11.3%</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>-51.2%</t>
+          <t>-26.7%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>169060</v>
+        <v>164830</v>
       </c>
       <c r="B8" t="n">
-        <v>99272</v>
+        <v>215325</v>
       </c>
       <c r="C8" t="n">
-        <v>164470</v>
+        <v>149948</v>
       </c>
       <c r="D8" t="n">
-        <v>67971</v>
+        <v>137644</v>
       </c>
       <c r="E8" t="n">
-        <v>3626873</v>
+        <v>3941651</v>
       </c>
       <c r="F8" t="n">
-        <v>893114</v>
+        <v>1235180</v>
       </c>
       <c r="G8" t="n">
-        <v>1809</v>
+        <v>1967</v>
       </c>
       <c r="H8" t="n">
-        <v>2374</v>
+        <v>2686</v>
       </c>
       <c r="I8" t="n">
-        <v>1734</v>
+        <v>1601</v>
       </c>
       <c r="J8" t="n">
-        <v>1579</v>
+        <v>2533</v>
       </c>
       <c r="K8" t="n">
-        <v>-23.79949452401011</v>
+        <v>-26.76842889054356</v>
       </c>
       <c r="L8" t="n">
-        <v>9.816339455351496</v>
+        <v>-36.79431504145282</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>70.3%</t>
+          <t>-23.5%</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>142.0%</t>
+          <t>8.9%</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>306.1%</t>
+          <t>219.1%</t>
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.01070034307346504</v>
+        <v>0.01193350724989383</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.02391409460875171</v>
+        <v>0.01247416695692558</v>
       </c>
       <c r="R8" t="n">
-        <v>0.01054295616221803</v>
+        <v>0.01067703470536453</v>
       </c>
       <c r="S8" t="n">
-        <v>0.02323049535831458</v>
+        <v>0.0184025456975967</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>-55.3%</t>
+          <t>-4.3%</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>-54.6%</t>
+          <t>-42.0%</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>154442</v>
+        <v>140165</v>
       </c>
       <c r="B9" t="n">
-        <v>119543</v>
+        <v>137891</v>
       </c>
       <c r="C9" t="n">
-        <v>160345</v>
+        <v>133822</v>
       </c>
       <c r="D9" t="n">
-        <v>117574</v>
+        <v>125551</v>
       </c>
       <c r="E9" t="n">
-        <v>2898422</v>
+        <v>3172409</v>
       </c>
       <c r="F9" t="n">
-        <v>2622645</v>
+        <v>2884256</v>
       </c>
       <c r="G9" t="n">
-        <v>5500</v>
+        <v>5603</v>
       </c>
       <c r="H9" t="n">
-        <v>6430</v>
+        <v>6505</v>
       </c>
       <c r="I9" t="n">
-        <v>5490</v>
+        <v>4999</v>
       </c>
       <c r="J9" t="n">
-        <v>6246</v>
+        <v>5997</v>
       </c>
       <c r="K9" t="n">
-        <v>-14.46345256609643</v>
+        <v>-13.86625672559569</v>
       </c>
       <c r="L9" t="n">
-        <v>-12.10374639769453</v>
+        <v>-16.64165416041354</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>29.2%</t>
+          <t>1.6%</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>36.4%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>10.5%</t>
+          <t>10.0%</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>0.0356120744357105</v>
+        <v>0.03997431598473228</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.05378817663936826</v>
+        <v>0.04717494252706848</v>
       </c>
       <c r="R9" t="n">
-        <v>0.03423867286164208</v>
+        <v>0.03735559175621347</v>
       </c>
       <c r="S9" t="n">
-        <v>0.05312398999778863</v>
+        <v>0.04776544989685466</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>-33.8%</t>
+          <t>-15.3%</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>-35.5%</t>
+          <t>-21.8%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2185947</v>
+        <v>2195962</v>
       </c>
       <c r="B10" t="n">
-        <v>1849274</v>
+        <v>2106220</v>
       </c>
       <c r="C10" t="n">
-        <v>2206240</v>
+        <v>2065119</v>
       </c>
       <c r="D10" t="n">
-        <v>1775141</v>
+        <v>1887398</v>
       </c>
       <c r="E10" t="n">
-        <v>43684570</v>
+        <v>47953674</v>
       </c>
       <c r="F10" t="n">
-        <v>36576317</v>
+        <v>40540741</v>
       </c>
       <c r="G10" t="n">
-        <v>92076</v>
+        <v>93924</v>
       </c>
       <c r="H10" t="n">
-        <v>90757</v>
+        <v>94821</v>
       </c>
       <c r="I10" t="n">
-        <v>92758</v>
+        <v>85036</v>
       </c>
       <c r="J10" t="n">
-        <v>91232</v>
+        <v>87328</v>
       </c>
       <c r="K10" t="n">
-        <v>1.45333142347146</v>
+        <v>-0.9459929762394403</v>
       </c>
       <c r="L10" t="n">
-        <v>1.672658716239916</v>
+        <v>-2.624587761084651</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>4.3%</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>24.3%</t>
+          <t>9.4%</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>19.4%</t>
+          <t>18.3%</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.04212178977806873</v>
+        <v>0.0427712319247783</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.04907709728250113</v>
+        <v>0.04501951363105468</v>
       </c>
       <c r="R10" t="n">
-        <v>0.04204347668431358</v>
+        <v>0.04117728808848304</v>
       </c>
       <c r="S10" t="n">
-        <v>0.05139422727546713</v>
+        <v>0.04626899043021133</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>-14.2%</t>
+          <t>-5.0%</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>-18.2%</t>
+          <t>-11.0%</t>
         </is>
       </c>
     </row>

</xml_diff>